<commit_message>
Expand COMS production mappings
</commit_message>
<xml_diff>
--- a/mappings/SSN2BFO-COMS.xlsx
+++ b/mappings/SSN2BFO-COMS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alecsculley/Documents/GitHub/SSN-to-BFO/mappings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B96C040-C977-1F4B-92B4-2ED8736B77A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{749F49C5-523B-4C4A-8A1A-4F21E744E901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15120" yWindow="660" windowWidth="15120" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34620" yWindow="1180" windowWidth="15120" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="162">
   <si>
     <t>sssom:subject_id</t>
   </si>
@@ -336,13 +336,184 @@
   </si>
   <si>
     <t>(sosa:Observation or sosa:Actuation or sosa:Sampling)</t>
+  </si>
+  <si>
+    <t>sosa:hasSample</t>
+  </si>
+  <si>
+    <t>owl:propertyChainAxiom</t>
+  </si>
+  <si>
+    <t>cco:represented_by o bfo:generically_depends_on</t>
+  </si>
+  <si>
+    <t>sosa:hosts</t>
+  </si>
+  <si>
+    <t>sosa:isHostedBy</t>
+  </si>
+  <si>
+    <t>bfo:bearer_of o bfo:has_realization o bfo:has_participant</t>
+  </si>
+  <si>
+    <t>bfo:participates_in o bfo:realizes o bfo:inheres_in</t>
+  </si>
+  <si>
+    <t>sosa:isActedOnBy</t>
+  </si>
+  <si>
+    <t>cco:is_affected_by</t>
+  </si>
+  <si>
+    <t>sosa:isObservedBy</t>
+  </si>
+  <si>
+    <t>sosa:observes</t>
+  </si>
+  <si>
+    <t>bfo:has_participant</t>
+  </si>
+  <si>
+    <t>bfo:participates_in</t>
+  </si>
+  <si>
+    <t>sosa:isResultOf</t>
+  </si>
+  <si>
+    <t>cco:is_output_of</t>
+  </si>
+  <si>
+    <t>sosa:isSampleOf</t>
+  </si>
+  <si>
+    <t>bfo:is_carrier_of o cco:represents</t>
+  </si>
+  <si>
+    <t>sosa:madeActuation</t>
+  </si>
+  <si>
+    <t>cco:agent_in</t>
+  </si>
+  <si>
+    <t>sosa:madeByActuator</t>
+  </si>
+  <si>
+    <t>sosa:madeBySampler</t>
+  </si>
+  <si>
+    <t>sosa:madeBySensor</t>
+  </si>
+  <si>
+    <t>sosa:madeObservation</t>
+  </si>
+  <si>
+    <t>cco:has_agent</t>
+  </si>
+  <si>
+    <t>sosa:madeSampling</t>
+  </si>
+  <si>
+    <t>sosa:observedProperty</t>
+  </si>
+  <si>
+    <t>cco:has_input</t>
+  </si>
+  <si>
+    <t>ssn-system:hasOperatingProperty</t>
+  </si>
+  <si>
+    <t>ssn-system:hasOperatingRange</t>
+  </si>
+  <si>
+    <t>ssn-system:hasSurvivalProperty</t>
+  </si>
+  <si>
+    <t>ssn-system:hasSurvivalRange</t>
+  </si>
+  <si>
+    <t>ssn-system:hasSystemCapability</t>
+  </si>
+  <si>
+    <t>bfo:bearer_of</t>
+  </si>
+  <si>
+    <t>ssn-system:hasSystemProperty</t>
+  </si>
+  <si>
+    <t>ssn:deployedOnPlatform</t>
+  </si>
+  <si>
+    <t>ssn:deployedSystem</t>
+  </si>
+  <si>
+    <t>ssn:detects</t>
+  </si>
+  <si>
+    <t>ssn:forProperty</t>
+  </si>
+  <si>
+    <t>ssn:hasDeployment</t>
+  </si>
+  <si>
+    <t>ssn:hasInput</t>
+  </si>
+  <si>
+    <t>ssn:hasOutput</t>
+  </si>
+  <si>
+    <t>ssn:hasProperty</t>
+  </si>
+  <si>
+    <t>ssn:hasSubSystem</t>
+  </si>
+  <si>
+    <t>ssn:implementedBy</t>
+  </si>
+  <si>
+    <t>ssn:implements</t>
+  </si>
+  <si>
+    <t>ssn:inDeployment</t>
+  </si>
+  <si>
+    <t>ssn:isProxyFor</t>
+  </si>
+  <si>
+    <t>ssn:wasOriginatedBy</t>
+  </si>
+  <si>
+    <t>bfo:has_continuant_part</t>
+  </si>
+  <si>
+    <t>cco:process_started_by</t>
+  </si>
+  <si>
+    <t>cco:prescribes</t>
+  </si>
+  <si>
+    <t>cco:described_by o cco:is_about</t>
+  </si>
+  <si>
+    <t>(ssn-system:SystemCapability or ssn-system:OperatingRange or ssn-system:SurvivalRange)</t>
+  </si>
+  <si>
+    <t>bfo:occupies_temporal_region</t>
+  </si>
+  <si>
+    <t>sosa:Sensor</t>
+  </si>
+  <si>
+    <t>bfo:MaterialEntity and (bfo:bearer_of some (bfo:RealizableEntity and (bfo:has_realization some sosa:Observation))) and (cco:agent_in some sosa:Observation)</t>
+  </si>
+  <si>
+    <t>bfo:specifically_depended_on_by</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -359,16 +530,26 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -391,11 +572,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -405,6 +612,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -619,7 +832,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.5" style="3" customWidth="1"/>
@@ -1042,80 +1255,91 @@
         <v>85</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" ht="85" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B38" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C38" s="3" t="s">
+      <c r="B39" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="85" x14ac:dyDescent="0.2">
-      <c r="A39" s="3" t="s">
+    <row r="40" spans="1:3" ht="85" x14ac:dyDescent="0.2">
+      <c r="A40" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B40" t="s">
         <v>11</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C40" s="3" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A40" s="3" t="s">
+    <row r="41" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A41" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B40" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C40" s="3" t="s">
+      <c r="B41" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C41" s="3" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A41" s="3" t="s">
+    <row r="42" spans="1:3" ht="119" x14ac:dyDescent="0.2">
+      <c r="A42" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B41" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C41" s="3" t="s">
+      <c r="B42" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42" s="3" t="s">
         <v>93</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="85" x14ac:dyDescent="0.2">
-      <c r="A42" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="85" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="85" x14ac:dyDescent="0.2">
+      <c r="A44" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B43" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C43" s="3" t="s">
+      <c r="B44" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C44" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="68" x14ac:dyDescent="0.2">
-      <c r="A44" s="3" t="s">
+    <row r="45" spans="1:3" ht="68" x14ac:dyDescent="0.2">
+      <c r="A45" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B44" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C44" s="3" t="s">
+      <c r="B45" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C45" s="3" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1126,12 +1350,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.1640625" customWidth="1"/>
     <col min="2" max="2" width="26.1640625" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="3" max="3" width="44.5" customWidth="1"/>
     <col min="4" max="4" width="43.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1252,6 +1476,12 @@
       <c r="A11" s="4" t="s">
         <v>77</v>
       </c>
+      <c r="B11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
@@ -1268,6 +1498,12 @@
       <c r="A13" s="4" t="s">
         <v>80</v>
       </c>
+      <c r="B13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
@@ -1283,6 +1519,496 @@
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>82</v>
+      </c>
+      <c r="B15" t="s">
+        <v>102</v>
+      </c>
+      <c r="C15" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C16" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B17" t="s">
+        <v>106</v>
+      </c>
+      <c r="C17" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B18" t="s">
+        <v>106</v>
+      </c>
+      <c r="C18" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C19" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B20" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B21" t="s">
+        <v>102</v>
+      </c>
+      <c r="C21" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B22" t="s">
+        <v>103</v>
+      </c>
+      <c r="C22" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B23" t="s">
+        <v>102</v>
+      </c>
+      <c r="C23" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B24" t="s">
+        <v>103</v>
+      </c>
+      <c r="C24" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B25" t="s">
+        <v>66</v>
+      </c>
+      <c r="C25" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B26" t="s">
+        <v>102</v>
+      </c>
+      <c r="C26" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B27" t="s">
+        <v>103</v>
+      </c>
+      <c r="C27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B28" t="s">
+        <v>102</v>
+      </c>
+      <c r="C28" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B29" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B30" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B31" t="s">
+        <v>66</v>
+      </c>
+      <c r="C31" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B32" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B33" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B34" t="s">
+        <v>102</v>
+      </c>
+      <c r="C34" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B35" t="s">
+        <v>103</v>
+      </c>
+      <c r="C35" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B36" t="s">
+        <v>66</v>
+      </c>
+      <c r="C36" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="B37" t="s">
+        <v>66</v>
+      </c>
+      <c r="C37" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>133</v>
+      </c>
+      <c r="B38" t="s">
+        <v>66</v>
+      </c>
+      <c r="C38" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>134</v>
+      </c>
+      <c r="B39" t="s">
+        <v>66</v>
+      </c>
+      <c r="C39" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>135</v>
+      </c>
+      <c r="B40" t="s">
+        <v>66</v>
+      </c>
+      <c r="C40" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>136</v>
+      </c>
+      <c r="B41" t="s">
+        <v>66</v>
+      </c>
+      <c r="C41" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>138</v>
+      </c>
+      <c r="B42" t="s">
+        <v>66</v>
+      </c>
+      <c r="C42" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>139</v>
+      </c>
+      <c r="B43" t="s">
+        <v>66</v>
+      </c>
+      <c r="C43" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>140</v>
+      </c>
+      <c r="B44" t="s">
+        <v>66</v>
+      </c>
+      <c r="C44" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>141</v>
+      </c>
+      <c r="B45" t="s">
+        <v>66</v>
+      </c>
+      <c r="C45" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>142</v>
+      </c>
+      <c r="B46" t="s">
+        <v>106</v>
+      </c>
+      <c r="C46" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>143</v>
+      </c>
+      <c r="B47" t="s">
+        <v>66</v>
+      </c>
+      <c r="C47" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>144</v>
+      </c>
+      <c r="B48" t="s">
+        <v>102</v>
+      </c>
+      <c r="C48" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>144</v>
+      </c>
+      <c r="B49" t="s">
+        <v>103</v>
+      </c>
+      <c r="C49" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>145</v>
+      </c>
+      <c r="B50" t="s">
+        <v>102</v>
+      </c>
+      <c r="C50" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>145</v>
+      </c>
+      <c r="B51" t="s">
+        <v>103</v>
+      </c>
+      <c r="C51" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>146</v>
+      </c>
+      <c r="B52" t="s">
+        <v>103</v>
+      </c>
+      <c r="C52" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>147</v>
+      </c>
+      <c r="B53" t="s">
+        <v>66</v>
+      </c>
+      <c r="C53" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>148</v>
+      </c>
+      <c r="B54" t="s">
+        <v>66</v>
+      </c>
+      <c r="C54" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>149</v>
+      </c>
+      <c r="B55" t="s">
+        <v>66</v>
+      </c>
+      <c r="C55" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>150</v>
+      </c>
+      <c r="B56" t="s">
+        <v>66</v>
+      </c>
+      <c r="C56" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>151</v>
+      </c>
+      <c r="B57" t="s">
+        <v>102</v>
+      </c>
+      <c r="C57" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>151</v>
+      </c>
+      <c r="B58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C58" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>152</v>
+      </c>
+      <c r="B59" t="s">
+        <v>66</v>
+      </c>
+      <c r="C59" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replace system bearer mappings with typing coverage
</commit_message>
<xml_diff>
--- a/mappings/SSN2BFO-COMS.xlsx
+++ b/mappings/SSN2BFO-COMS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alecsculley/Documents/GitHub/SSN-to-BFO/mappings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{749F49C5-523B-4C4A-8A1A-4F21E744E901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00A6B318-973F-1345-98D6-FFBAA65AA06D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34620" yWindow="1180" windowWidth="15120" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34620" yWindow="1180" windowWidth="18560" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="161">
   <si>
     <t>sssom:subject_id</t>
   </si>
@@ -432,9 +432,6 @@
   </si>
   <si>
     <t>ssn-system:hasSystemCapability</t>
-  </si>
-  <si>
-    <t>bfo:bearer_of</t>
   </si>
   <si>
     <t>ssn-system:hasSystemProperty</t>
@@ -1257,13 +1254,13 @@
     </row>
     <row r="38" spans="1:3" ht="85" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>159</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="34" x14ac:dyDescent="0.2">
@@ -1350,7 +1347,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.1640625" customWidth="1"/>
@@ -1480,7 +1477,7 @@
         <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -1502,7 +1499,7 @@
         <v>102</v>
       </c>
       <c r="C13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -1601,7 +1598,7 @@
         <v>103</v>
       </c>
       <c r="C22" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -1612,7 +1609,7 @@
         <v>102</v>
       </c>
       <c r="C23" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -1722,7 +1719,7 @@
         <v>103</v>
       </c>
       <c r="C33" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -1733,7 +1730,7 @@
         <v>102</v>
       </c>
       <c r="C34" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -1766,7 +1763,7 @@
         <v>66</v>
       </c>
       <c r="C37" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -1774,241 +1771,274 @@
         <v>133</v>
       </c>
       <c r="B38" t="s">
-        <v>66</v>
+        <v>102</v>
       </c>
       <c r="C38" t="s">
-        <v>137</v>
+        <v>63</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B39" t="s">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="C39" t="s">
-        <v>161</v>
+        <v>41</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B40" t="s">
         <v>66</v>
       </c>
       <c r="C40" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B41" t="s">
-        <v>66</v>
+        <v>102</v>
       </c>
       <c r="C41" t="s">
-        <v>137</v>
+        <v>63</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B42" t="s">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="C42" t="s">
-        <v>161</v>
+        <v>96</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B43" t="s">
-        <v>66</v>
+        <v>102</v>
       </c>
       <c r="C43" t="s">
-        <v>116</v>
+        <v>63</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B44" t="s">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="C44" t="s">
-        <v>116</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B45" t="s">
         <v>66</v>
       </c>
       <c r="C45" t="s">
-        <v>113</v>
+        <v>160</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B46" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="C46" t="s">
-        <v>156</v>
+        <v>116</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B47" t="s">
         <v>66</v>
       </c>
       <c r="C47" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B48" t="s">
-        <v>102</v>
+        <v>66</v>
       </c>
       <c r="C48" t="s">
-        <v>86</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B49" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C49" t="s">
-        <v>57</v>
+        <v>155</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B50" t="s">
-        <v>102</v>
+        <v>66</v>
       </c>
       <c r="C50" t="s">
-        <v>86</v>
+        <v>117</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B51" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C51" t="s">
-        <v>58</v>
+        <v>86</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B52" t="s">
         <v>103</v>
       </c>
       <c r="C52" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B53" t="s">
-        <v>66</v>
+        <v>102</v>
       </c>
       <c r="C53" t="s">
-        <v>153</v>
+        <v>86</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B54" t="s">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="C54" t="s">
-        <v>155</v>
+        <v>58</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B55" t="s">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="C55" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B56" t="s">
         <v>66</v>
       </c>
       <c r="C56" t="s">
-        <v>117</v>
+        <v>152</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B57" t="s">
-        <v>102</v>
+        <v>66</v>
       </c>
       <c r="C57" t="s">
-        <v>61</v>
+        <v>154</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B58" t="s">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="C58" t="s">
-        <v>59</v>
+        <v>79</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B59" t="s">
         <v>66</v>
       </c>
       <c r="C59" t="s">
-        <v>154</v>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>150</v>
+      </c>
+      <c r="B60" t="s">
+        <v>102</v>
+      </c>
+      <c r="C60" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>150</v>
+      </c>
+      <c r="B61" t="s">
+        <v>103</v>
+      </c>
+      <c r="C61" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>151</v>
+      </c>
+      <c r="B62" t="s">
+        <v>66</v>
+      </c>
+      <c r="C62" t="s">
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Defer sample property chains for OWL 2 DL simplicity
</commit_message>
<xml_diff>
--- a/mappings/SSN2BFO-COMS.xlsx
+++ b/mappings/SSN2BFO-COMS.xlsx
@@ -1783,14 +1783,9 @@
           <t>sosa:hasSample</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>owl:propertyChainAxiom</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>cco:represented_by o bfo:generically_depends_on</t>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Property-chain mapping deferred because an owl:propertyChainAxiom makes sosa:hasSample non-simple, which conflicts with the pinned SOSA/SSN inverse-functional declaration. The source ontology remains unchanged; the representation intent belongs in a rule, SHACL, or annotation layer rather than the OWL 2 DL mapping product.</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -1805,14 +1800,9 @@
           <t>sosa:isSampleOf</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>owl:propertyChainAxiom</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>bfo:is_carrier_of o cco:represents</t>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Property-chain mapping deferred because an owl:propertyChainAxiom makes sosa:isSampleOf non-simple, which conflicts with the pinned SOSA/SSN functional declaration and the minimum-cardinality restriction on sosa:Sample. The source ontology remains unchanged; the representation intent belongs in a rule, SHACL, or annotation layer rather than the OWL 2 DL mapping product.</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">

</xml_diff>